<commit_message>
Only 4 companies actually uploaded
</commit_message>
<xml_diff>
--- a/master_list.xlsx
+++ b/master_list.xlsx
@@ -1,22 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grego\OneDrive\Desktop\Project_Scrape\2025\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\grego\Desktop\SFCR_using_Mistral_2025-main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCBC56DA-995A-422B-B3BE-34324DF0EA7B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{062FA2B5-F525-47B1-AAED-7F47290B5687}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4400" yWindow="4110" windowWidth="19200" windowHeight="11170" xr2:uid="{1F6F973B-83FC-459C-AE8F-1356A634A5E2}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="19095" windowHeight="12075" xr2:uid="{1F6F973B-83FC-459C-AE8F-1356A634A5E2}"/>
   </bookViews>
   <sheets>
-    <sheet name="ITALY_2024" sheetId="1" r:id="rId1"/>
+    <sheet name="ITALY_2025" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ITALY_2024!$A$1:$F$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">ITALY_2025!$A$1:$F$34</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -209,9 +209,6 @@
     <t>SFCR 2024 CREDEMVITA.pdf</t>
   </si>
   <si>
-    <t>2024.12 QRT SFCR AXA MPS Assicurazioni Vita.pdf</t>
-  </si>
-  <si>
     <t>ca_vita_sfcr_2024.pdf</t>
   </si>
   <si>
@@ -224,15 +221,9 @@
     <t>Mediolanum_Vita_Relazione_Unica_2024.pdf</t>
   </si>
   <si>
-    <t>2024 Relazione sulla Solvibilita e Condizione Finanziaria Generali Italia.pdf</t>
-  </si>
-  <si>
     <t>Fascicolo-SFCR_2024_BBPMV-signed_con-opinion.pdf</t>
   </si>
   <si>
-    <t>HDI Assicurazioni S.p.A. - Avviso pubblicazione SFCR - IT.pdf</t>
-  </si>
-  <si>
     <t>relazioneunicasolvibilita_condizionefinanziaria_31122024.pdf</t>
   </si>
   <si>
@@ -242,9 +233,6 @@
     <t>SFCR_2024_CNP_Vita_Assicura_con_Relazione.pdf</t>
   </si>
   <si>
-    <t>SFCR_G0010_20241231.pdf</t>
-  </si>
-  <si>
     <t>SFCR_Annex_Helvetia Vita_2024.pdf</t>
   </si>
   <si>
@@ -257,9 +245,6 @@
     <t>UAV_Fascicolo_SFCR_2024_con_relazioni_PwC.pdf</t>
   </si>
   <si>
-    <t>zil_scfr_2024_web.pdf</t>
-  </si>
-  <si>
     <t>S_02_01_02_A</t>
   </si>
   <si>
@@ -288,6 +273,21 @@
   </si>
   <si>
     <t>CREDEM_VITA</t>
+  </si>
+  <si>
+    <t>2025 Relazione sulla Solvibilita e Condizione Finanziaria Generali Italia.pdf</t>
+  </si>
+  <si>
+    <t>Fascicolo AMAV_SFCR_31.12.2025_SITO.pdf</t>
+  </si>
+  <si>
+    <t>SFCR_G0010_20251231.pdf</t>
+  </si>
+  <si>
+    <t>SFCR2025EN.pdf</t>
+  </si>
+  <si>
+    <t>zil_sfcr_2025_web.pdf</t>
   </si>
 </sst>
 </file>
@@ -303,12 +303,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -323,9 +329,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="1" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -661,20 +669,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F43813C6-155E-442B-992A-28BDB54378D4}">
   <dimension ref="A1:F34"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="2" width="31.1796875" customWidth="1"/>
-    <col min="3" max="3" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="78.90625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.54296875" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="31.19921875" customWidth="1"/>
+    <col min="3" max="3" width="16.19921875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="78.9296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.53125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -689,663 +697,663 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C2" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="D2" t="s">
         <v>55</v>
       </c>
       <c r="E2" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F2" s="1">
         <v>197</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C3" t="s">
         <v>77</v>
-      </c>
-      <c r="C3" t="s">
-        <v>82</v>
       </c>
       <c r="D3" t="s">
         <v>55</v>
       </c>
       <c r="E3" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F3" s="1">
         <v>198</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A4" t="s">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B4" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="D4" t="s">
-        <v>56</v>
-      </c>
-      <c r="E4" t="s">
-        <v>73</v>
-      </c>
-      <c r="F4" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="D4" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F4" s="3">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>9</v>
       </c>
       <c r="B5" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C5" t="s">
         <v>11</v>
       </c>
       <c r="D5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E5" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F5" s="1">
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C6" t="s">
         <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="E6" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F6" s="1">
         <v>62</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>12</v>
       </c>
       <c r="B7" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C7" t="s">
         <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E7" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F7" s="1">
         <v>158</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>13</v>
       </c>
       <c r="B8" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C8" t="s">
         <v>14</v>
       </c>
       <c r="D8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E8" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F8" s="1">
         <v>159</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="C9" t="s">
         <v>16</v>
       </c>
       <c r="D9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E9" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F9" s="1">
         <v>106</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>18</v>
       </c>
       <c r="B10" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C10" t="s">
         <v>17</v>
       </c>
       <c r="D10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E10" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F10" s="1">
         <v>164</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>19</v>
       </c>
       <c r="B11" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C11" t="s">
         <v>17</v>
       </c>
       <c r="D11" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="E11" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F11" s="1">
         <v>165</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A12" t="s">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A12" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B12" t="s">
-        <v>79</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="B12" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D12" t="s">
-        <v>61</v>
-      </c>
-      <c r="E12" t="s">
-        <v>73</v>
-      </c>
-      <c r="F12" s="1">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A13" t="s">
+      <c r="D12" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F12" s="3">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A13" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B13" t="s">
-        <v>80</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="B13" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D13" t="s">
-        <v>61</v>
-      </c>
-      <c r="E13" t="s">
-        <v>74</v>
-      </c>
-      <c r="F13" s="1">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="D13" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" s="3">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>34</v>
       </c>
       <c r="B14" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C14" t="s">
         <v>21</v>
       </c>
       <c r="D14" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E14" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F14" s="1">
         <v>80</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C15" t="s">
         <v>21</v>
       </c>
       <c r="D15" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E15" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F15" s="1">
         <v>81</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A16" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B16" t="s">
-        <v>79</v>
-      </c>
-      <c r="C16" t="s">
+      <c r="B16" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D16" t="s">
-        <v>63</v>
-      </c>
-      <c r="E16" t="s">
-        <v>73</v>
-      </c>
-      <c r="F16" s="1">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17" t="s">
+      <c r="D16" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F16" s="3">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A17" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B17" t="s">
-        <v>80</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="B17" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D17" t="s">
-        <v>63</v>
-      </c>
-      <c r="E17" t="s">
-        <v>74</v>
-      </c>
-      <c r="F17" s="1">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="D17" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F17" s="3">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>38</v>
       </c>
       <c r="B18" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C18" t="s">
         <v>23</v>
       </c>
       <c r="D18" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E18" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F18" s="1">
         <v>136</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C19" t="s">
         <v>23</v>
       </c>
       <c r="D19" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="E19" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F19" s="1">
         <v>137</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>40</v>
       </c>
       <c r="B20" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C20" t="s">
         <v>24</v>
       </c>
       <c r="D20" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E20" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F20" s="1">
         <v>250</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>41</v>
       </c>
       <c r="B21" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C21" t="s">
         <v>24</v>
       </c>
       <c r="D21" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E21" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F21" s="1">
         <v>251</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>42</v>
       </c>
       <c r="B22" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C22" t="s">
         <v>25</v>
       </c>
       <c r="D22" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E22" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F22" s="1">
         <v>116</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>43</v>
       </c>
       <c r="B23" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C23" t="s">
         <v>25</v>
       </c>
       <c r="D23" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E23" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F23" s="1">
         <v>117</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>44</v>
       </c>
       <c r="B24" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C24" t="s">
         <v>26</v>
       </c>
       <c r="D24" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="E24" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F24" s="1">
         <v>233</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>45</v>
       </c>
       <c r="B25" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C25" t="s">
         <v>26</v>
       </c>
       <c r="D25" t="s">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="E25" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F25" s="1">
         <v>234</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>46</v>
       </c>
       <c r="B26" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="C26" t="s">
         <v>27</v>
       </c>
       <c r="D26" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E26" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F26" s="1">
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>47</v>
       </c>
       <c r="B27" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="C27" t="s">
         <v>27</v>
       </c>
       <c r="D27" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="E27" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F27" s="1">
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>48</v>
       </c>
       <c r="B28" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C28" t="s">
         <v>28</v>
       </c>
       <c r="D28" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E28" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F28" s="1">
         <v>93</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>49</v>
       </c>
       <c r="B29" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C29" t="s">
         <v>28</v>
       </c>
       <c r="D29" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="E29" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F29" s="1">
         <v>94</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>50</v>
       </c>
       <c r="B30" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="C30" t="s">
         <v>29</v>
       </c>
       <c r="D30" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="E30" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F30" s="1">
         <v>71</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>51</v>
       </c>
       <c r="B31" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="C31" t="s">
         <v>30</v>
       </c>
       <c r="D31" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E31" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="F31" s="1">
         <v>110</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>52</v>
       </c>
       <c r="B32" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="C32" t="s">
         <v>30</v>
       </c>
       <c r="D32" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="E32" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="F32" s="1">
         <v>111</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A33" t="s">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A33" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B33" t="s">
-        <v>79</v>
-      </c>
-      <c r="C33" t="s">
+      <c r="B33" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D33" t="s">
-        <v>72</v>
-      </c>
-      <c r="E33" t="s">
-        <v>73</v>
-      </c>
-      <c r="F33" s="1">
+      <c r="D33" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="F33" s="3">
         <v>58</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A34" t="s">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A34" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B34" t="s">
-        <v>80</v>
-      </c>
-      <c r="C34" t="s">
+      <c r="B34" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D34" t="s">
-        <v>72</v>
-      </c>
-      <c r="E34" t="s">
-        <v>74</v>
-      </c>
-      <c r="F34" s="1">
+      <c r="D34" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="E34" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F34" s="3">
         <v>59</v>
       </c>
     </row>

</xml_diff>